<commit_message>
mise à jour du copilote recrutement
</commit_message>
<xml_diff>
--- a/tests/fixtures/agent2_v2/tableau_comparaison_agent2.xlsx
+++ b/tests/fixtures/agent2_v2/tableau_comparaison_agent2.xlsx
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Le candidat maitrise l'ensemble des competences techniques requises, notamment Python, Machine Learning, SQL, scikit-learn, TensorFlow, PyTorch, Docker, Git et le developpement de pipelines de donnees.</t>
+          <t>Couverture totale des compétences techniques et transversales requises par l'offre.</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Toutes les competences transversales demandees sont validees (travail en equipe, communication, autonomie, resolution de problemes, gestion de projet).</t>
+          <t>Maîtrise parfaite des langues demandées (Français et Anglais professionnel).</t>
         </is>
       </c>
     </row>
@@ -1225,27 +1225,27 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Les exigences linguistiques sont parfaitement remplies avec la maitrise du francais et de l'anglais professionnel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>L'experience du candidat (13 ans) depasse largement le minimum requis de 5 ans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49"/>
+          <t>Expérience solide de 13 ans qui surpasse largement le minimum de 5 ans exigé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>7. POINTS MANQUANTS</t>
+        </is>
+      </c>
+    </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>7. POINTS MANQUANTS</t>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Aucune compétence ni langue requise ne manque au profil.</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
     <row r="53" ht="80" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>Le candidat obtient un score de compatibilite de 100/100 en raison de la couverture integrale des competences techniques et transversales requises, de la maitrise des langues demandees et d'une experience de 13 ans qui depasse le seuil minimum de 5 ans.</t>
+          <t>Le score de compatibilité de 100/100 s'explique par une adéquation parfaite : l'intégralité des compétences techniques, transversales et linguistiques requises est couverte par le profil, et l'expérience de 13 ans dépasse amplement les 5 ans minimum demandés.</t>
         </is>
       </c>
     </row>
@@ -1269,12 +1269,12 @@
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A50:E50"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="A52:E52"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise des compétences techniques clés telles que Python, Machine Learning, SQL, scikit-learn, le traitement et l'analyse de données, ainsi que Git.</t>
+          <t>Solide maîtrise des compétences techniques de base incluant Python, Machine Learning, SQL, scikit-learn, le traitement et l'analyse de données, Git et le développement de pipelines de données.</t>
         </is>
       </c>
     </row>
@@ -2023,27 +2023,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Bonne couverture des compétences transversales et linguistiques avec le travail en équipe, la communication, le français et l'anglais professionnel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47"/>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+          <t>Bonne adéquation sur le plan des compétences comportementales avec la maîtrise du travail en équipe et de la communication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Maîtrise totale des langues requises (Français et Anglais professionnel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>7. POINTS MANQUANTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Absence de compétences requises en deep learning (TensorFlow, PyTorch) et en conteneurisation (Docker).</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Manque de compétences transversales recherchées telles que l'autonomie, la résolution de problèmes et la gestion de projet.</t>
+          <t>Absence des compétences en deep learning et conteneurisation demandées, notamment TensorFlow, PyTorch et Docker.</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Expérience de 3 ans inférieure aux 5 ans d'expérience minimum requis par l'offre.</t>
+          <t>Manque des compétences transversales attendues telles que l'autonomie, la résolution de problèmes et la gestion de projet.</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
     <row r="54" ht="80" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>Le candidat obtient un score de compatibilité de 69/100 (niveau : Bon). Ce score reflète une très bonne adéquation sur les compétences techniques fondamentales (Python, SQL, Machine Learning) et les langues, mais il est pondéré par l'écart sur l'expérience requise (3 ans contre 5 ans) et l'absence de certains outils avancés comme TensorFlow, PyTorch et Docker.</t>
+          <t>Le candidat obtient un score de 69 sur 100, correspondant à un niveau bon. Ce résultat reflète une couverture satisfaisante des compétences techniques et linguistiques essentielles, mais est tempéré par l'écart d'expérience (3 ans d'expérience relevés face aux 5 ans minimum exigés par l'offre) ainsi que par l'absence de certains outils avancés (TensorFlow, PyTorch, Docker) et de quelques compétences transversales.</t>
         </is>
       </c>
     </row>
@@ -2091,12 +2091,12 @@
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A48:E48"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise du SQL, du traitement et de l'analyse de données</t>
+          <t>Le candidat maitrise des competences cles telles que le SQL, le traitement et l'analyse de donnees.</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Solides compétences en travail en équipe, communication et gestion de projet</t>
+          <t>Il possede de solides competences transversales incluant le travail en equipe, la communication et la gestion de projet.</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise totale des langues requises (Français et Anglais professionnel)</t>
+          <t>Il maitrise le français et l'anglais professionnel.</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Expérience significative de 14 ans, dépassant largement le minimum requis de 5 ans</t>
+          <t>Il dispose de 14 ans d'experience, ce qui depasse largement le minimum de 5 ans requis.</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Absence des compétences techniques en Python, Machine Learning, scikit-learn, TensorFlow, PyTorch, Docker, Git et développement de pipelines de données</t>
+          <t>Absence de competences techniques essentielles pour le poste : Python, Machine Learning, scikit-learn, TensorFlow, PyTorch, Docker, Git et le developpement de pipelines de donnees.</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Absence des compétences transversales d'Autonomie et de Résolution de problèmes</t>
+          <t>Manque de competences comportementales requises : autonomie et resolution de problemes.</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
     <row r="55" ht="80" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>Le candidat obtient un score de compatibilité de 50/100 (niveau : Moyen). Bien que le candidat surpasse l'expérience requise (14 ans contre 5 ans minimum) et possède une bonne maîtrise des langues ainsi que quelques compétences de base (SQL, traitement et analyse de données, et soft skills associées), il lui manque des compétences techniques majeures exigées pour ce poste de Machine Learning Engineer / Data Scientist (Python, ML, frameworks associés, MLOps). Un cap anti-inflation a été appliqué, plafonnant le score à 50/100 en raison de l'inadéquation partielle des compétences techniques fondamentales pour le poste.</t>
+          <t>Le candidat obtient un score de compatibilite de 50 sur 100 (niveau moyen). Bien que son experience de 14 ans depasse l'exigence de l'offre et qu'il couvre plusieurs competences et les langues requises, il lui manque des competences techniques fondamentales pour ce poste en IA (Python, Machine Learning, frameworks associes, outils de developpement). En raison de ces lacunes techniques majeures, un cap anti-inflation a ete applique, plafonnant le score a 50 sur 100.</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Excellente maîtrise de Python, de SQL, du traitement et de l'analyse de données ainsi que du développement de pipelines de données.</t>
+          <t>Bonne maîtrise de Python, SQL, et des compétences en traitement, analyse de données et développement de pipelines de données.</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Compétences transversales solides incluant le travail en équipe, la communication, l'autonomie et la résolution de problèmes.</t>
+          <t>Excellentes compétences transversales validées (travail en équipe, communication, autonomie, résolution de problèmes).</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise totale des langues requises : Français et Anglais professionnel.</t>
+          <t>Maîtrise parfaite du français et bon niveau d'anglais professionnel.</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Expérience de 7 ans, dépassant les 5 ans minimum requis par l'offre.</t>
+          <t>Expérience solide de 7 ans, dépassant les 5 ans minimum requis par l'offre.</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Absence de compétences en Machine Learning, notamment scikit-learn, TensorFlow et PyTorch.</t>
+          <t>Absence des compétences en Machine Learning requises (Machine Learning, scikit-learn, TensorFlow, PyTorch).</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Manque de maîtrise des outils techniques demandés tels que Docker et Git.</t>
+          <t>Manque d'outils de versioning et conteneurisation demandés (Docker, Git).</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
     <row r="56" ht="80" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>Le score de 78/100 (niveau Très bon) s'explique par une forte adéquation sur les compétences fondamentales (Python, SQL, traitement des données), une maîtrise parfaite des langues requises et une expérience de 7 ans supérieure aux 5 ans exigés. Le retrait de points provient exclusivement des lacunes sur les compétences spécifiques au Machine Learning et aux outils de déploiement demandés dans l'offre.</t>
+          <t>Le candidat obtient un score de compatibilité de 78 sur 100 (niveau Très bon). Ce score s'explique par une solide couverture des compétences fondamentales en programmation et analyse (Python, SQL, traitement des données), d'excellentes aptitudes relationnelles, un profil linguistique parfaitement aligné, ainsi qu'une expérience de 7 ans supérieure aux exigences de l'offre (5 ans minimum). Cependant, le score est impacté par l'absence de compétences clés en Machine Learning et en ingénierie logicielle (scikit-learn, TensorFlow, PyTorch, Docker, Git, gestion de projet), qui étaient explicitement demandées pour ce poste de Machine Learning Engineer / Data Scientist.</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Excellente couverture des compétences techniques requises telles que Python, Machine Learning, SQL, scikit-learn, PyTorch, Docker, Git et le traitement de données.</t>
+          <t>Forte couverture des competences techniques requises incluant Python, Machine Learning, SQL, scikit-learn, PyTorch, Docker, Git, le traitement et l'analyse de donnees ainsi que le developpement de pipelines.</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise des compétences transversales clés incluant le travail en équipe, la communication, l'autonomie et la résolution de problèmes.</t>
+          <t>Maitrise des competences transversales demandees (Travail en equipe, Communication, Autonomie, Resolution de problemes).</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Maîtrise parfaite des langues demandées : Français et Anglais professionnel.</t>
+          <t>Maitrise complete des langues requises (Francais et Anglais professionnel).</t>
         </is>
       </c>
     </row>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Expérience de 8 ans, dépassant largement le minimum requis de 5 ans.</t>
+          <t>Experience solide de 8 ans superieure au minimum requis de 5 ans.</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Absence de la compétence technique TensorFlow.</t>
+          <t>Competence technique manquante : TensorFlow.</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Absence de la compétence transversale Gestion de projet.</t>
+          <t>Competence transversale manquante : Gestion de projet.</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
     <row r="55" ht="80" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>Le candidat obtient un score de compatibilité de 95 sur 100 (niveau Excellent). Ce résultat reflète une adéquation quasi-totale avec les exigences du poste, combinant une forte maîtrise des technologies clés (Python, PyTorch, scikit-learn, Docker), une expérience de 8 ans supérieure au minimum requis de 5 ans, ainsi qu'une couverture complète des langues. Seuls de légers manques sur TensorFlow et la gestion de projet préviennent l'obtention de la note maximale, sans compromettre la haute pertinence de la candidature.</t>
+          <t>Le candidat obtient un score de compatibilite de 95 sur 100, classe comme Excellent. Ce score reflete une adequation tres elevee avec le profil recherche grace a une excellente couverture des competences requises, une maitrise parfaite des langues et une experience de 8 ans depassant le minimum de 5 ans exige. Seules manquent les competences TensorFlow et Gestion de projet.</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Excellente couverture des competences techniques et transversales requises, notamment en Python, Machine Learning, SQL, scikit-learn, Docker, Git et en analyse de donnees.</t>
+          <t>Forte couverture des compétences techniques indispensables dont Python, Machine Learning, SQL, scikit-learn, Docker, Git, le traitement de données et les pipelines.</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5359,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Maitrise complete des langues demandees, a savoir le Francais et l'Anglais professionnel.</t>
+          <t>Maîtrise des aptitudes transversales requises incluant le travail en équipe, la communication, l'autonomie et la résolution de problèmes.</t>
         </is>
       </c>
     </row>
@@ -5371,27 +5371,27 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Experience solide de 9 ans, depassant largement le minimum requis de 5 ans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48"/>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+          <t>Maîtrise totale des langues requises (Français et Anglais professionnel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Expérience professionnelle de 9 ans, surpassant le minimum de 5 ans exigé par l'offre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>7. POINTS MANQUANTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Absence des competences en deep learning avec TensorFlow et PyTorch.</t>
         </is>
       </c>
     </row>
@@ -5403,36 +5403,48 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Absence de la competence transversale en Gestion de projet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52"/>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+          <t>Absence des frameworks de deep learning TensorFlow et PyTorch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Absence de la compétence en gestion de projet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>8. EXPLICATION</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="80" customHeight="1">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>Le candidat obtient un score de compatibilite de 92 sur 100 (niveau Excellent). Ce score reflete une tres forte adecuacion avec le poste, portee par une excellente maitrise des competences requises, une experience professionnelle de 9 ans superieure aux 5 ans exiges, ainsi qu'une parfaite couverture linguistique. Seules quelques lacunes sur des technologiques specifiques (TensorFlow, PyTorch) et la gestion de projet expliquent que le score ne soit pas maximal.</t>
+    <row r="55" ht="80" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>Le candidat obtient un score de compatibilité de 92 sur 100 qualifié d'Excellent. Ce score s'explique par une excellente adéquation du profil : une couverture quasi-totale des compétences techniques et transversales, une maîtrise parfaite des langues demandées et une expérience de 9 ans supérieure au seuil requis de 5 ans. Les seuls points d'écart concernent TensorFlow, PyTorch et la gestion de projet.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>